<commit_message>
carry1st: research (company, EBANX direct vs through Yuno, five LatAm markets, sources) and business-case model (xlsx + deck numbers + proposal text)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Carry1st/build/model/bc_model.xlsx
+++ b/Deals/Carry1st/build/model/bc_model.xlsx
@@ -1592,7 +1592,7 @@
       </c>
       <c r="G16" s="28" t="inlineStr">
         <is>
-          <t>ESTIMATE, range 3 to 6% of TPV. Anchors: dLocal FY2025 revenue / TPV = 2.68% (2.92% in 2024), a blended figure across pay-ins, pay-outs and very large merchants, so a floor for a $0.5 to 4.5M a month digital-goods merchant (FXC Intelligence, 26 Mar 2026, on dLocal's results of 18 Mar 2026). EBANX reviewer: about 5% per transaction plus a $200 monthly fee (Capterra, Nov 2021). FX spread of 1 to 3% on top of processing (Nuvei, 2026). Brazil IOF on FX 3.5% (Decree 12,466/2025, PayPro Global).</t>
+          <t>ESTIMATE, range 3 to 6% of TPV. Anchors: dLocal FY2025 revenue / TPV = 2.68% (2.92% in 2024), a blended figure across pay-ins, pay-outs and very large merchants, so a low anchor for a $0.5 to 4.5M a month digital-goods merchant (FXC Intelligence, 26 Mar 2026, on dLocal's results of 18 Mar 2026). EBANX reviewer: about 5% per transaction plus a $200 monthly fee (Capterra, Nov 2021). FX spread of 1 to 3% on top of processing (Nuvei, 2026). Brazil IOF on FX 3.5% (Decree 12,466/2025, PayPro Global).</t>
         </is>
       </c>
       <c r="H16" s="28" t="inlineStr">
@@ -1932,7 +1932,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1">
+    <row r="30" ht="15" customHeight="1">
       <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Annual maintenance, % of build cost per integration</t>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="G30" s="28" t="inlineStr">
         <is>
-          <t>Yuno estimate; 20 to 30% upkeep is the convention used in Yuno business cases (Luni, Oct 2026).</t>
+          <t>Yuno estimate; 20 to 30% upkeep is the convention used in Yuno business cases (Oct 2026).</t>
         </is>
       </c>
       <c r="H30" s="28" t="inlineStr"/>
@@ -2070,7 +2070,7 @@
     <row r="35" ht="15" customHeight="1">
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Tranche 1 · monthly TPV up to</t>
+          <t>Tranche 1 · monthly TPV ceiling</t>
         </is>
       </c>
       <c r="C35" s="26" t="inlineStr">
@@ -2136,7 +2136,7 @@
     <row r="37" ht="15" customHeight="1">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Tranche 2 · monthly TPV up to</t>
+          <t>Tranche 2 · monthly TPV ceiling</t>
         </is>
       </c>
       <c r="C37" s="26" t="inlineStr">
@@ -2427,7 +2427,7 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Tranche 1 · TPV up to</t>
+          <t>Tranche 1 · TPV ceiling</t>
         </is>
       </c>
       <c r="B7" s="44">
@@ -2449,7 +2449,7 @@
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Tranche 2 · TPV up to</t>
+          <t>Tranche 2 · TPV ceiling</t>
         </is>
       </c>
       <c r="B9" s="44">

</xml_diff>

<commit_message>
carry1st: time-to-market lever (run rate by mid 2027)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Carry1st/build/model/bc_model.xlsx
+++ b/Deals/Carry1st/build/model/bc_model.xlsx
@@ -13,8 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BreakEven" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ramp" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TimeToMarket" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -648,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1146,22 +1147,179 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="B28" s="23" t="inlineStr">
-        <is>
-          <t>How to read: Option A = EBANX direct at the baseline all-in cost (ESTIMATE until EBANX's quote replaces the baseline on Inputs). Option B = EBANX primary + dLocal second MoR through Yuno; its provider cost is the baseline minus the MDR reduction, plus Yuno's flat platform fee and usage in bps on the Net TPV above the included block. Levers: L1 MDR saving (100% contribution), L2 retries and routing, L3 local methods, L4 integrations avoided (per-market EBANX work, later direct integrations, maintenance; deck lever L2). Contribution view nets the take rate and processing cost on incremental GMV. Yuno-wide figures used only as guardrails: 7% authorization uplift, 30% recovered revenue (y.uno).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Time to market (L5, deck L3): 2027 value, kept apart</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Through Yuno: run-rate month</t>
+        </is>
+      </c>
+      <c r="D29" s="22">
+        <f>TimeToMarket!B23</f>
+        <v/>
+      </c>
+      <c r="E29" s="22">
+        <f>TimeToMarket!C23</f>
+        <v/>
+      </c>
+      <c r="F29" s="22">
+        <f>TimeToMarket!D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Extra sales in 2027</t>
+        </is>
+      </c>
+      <c r="D30" s="11">
+        <f>TimeToMarket!B24</f>
+        <v/>
+      </c>
+      <c r="E30" s="11">
+        <f>TimeToMarket!C24</f>
+        <v/>
+      </c>
+      <c r="F30" s="11">
+        <f>TimeToMarket!D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>L5 · 2027 value from reaching run rate sooner</t>
+        </is>
+      </c>
+      <c r="D31" s="16">
+        <f>TimeToMarket!B27</f>
+        <v/>
+      </c>
+      <c r="E31" s="16">
+        <f>TimeToMarket!C27</f>
+        <v/>
+      </c>
+      <c r="F31" s="16">
+        <f>TimeToMarket!D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>Recurring levers a year at run rate</t>
+        </is>
+      </c>
+      <c r="D32" s="11">
+        <f>TimeToMarket!B28</f>
+        <v/>
+      </c>
+      <c r="E32" s="11">
+        <f>TimeToMarket!C28</f>
+        <v/>
+      </c>
+      <c r="F32" s="11">
+        <f>TimeToMarket!D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>2027 value including time to market</t>
+        </is>
+      </c>
+      <c r="D33" s="16">
+        <f>TimeToMarket!B29</f>
+        <v/>
+      </c>
+      <c r="E33" s="16">
+        <f>TimeToMarket!C29</f>
+        <v/>
+      </c>
+      <c r="F33" s="16">
+        <f>TimeToMarket!D29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Net 2027 including time to market</t>
+        </is>
+      </c>
+      <c r="D34" s="16">
+        <f>TimeToMarket!B32</f>
+        <v/>
+      </c>
+      <c r="E34" s="16">
+        <f>TimeToMarket!C32</f>
+        <v/>
+      </c>
+      <c r="F34" s="16">
+        <f>TimeToMarket!D32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>2027 value / Yuno cost</t>
+        </is>
+      </c>
+      <c r="D35" s="20">
+        <f>TimeToMarket!B34</f>
+        <v/>
+      </c>
+      <c r="E35" s="20">
+        <f>TimeToMarket!C34</f>
+        <v/>
+      </c>
+      <c r="F35" s="20">
+        <f>TimeToMarket!D34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>How to read: Option A = EBANX direct at the baseline all-in cost (ESTIMATE until EBANX's quote replaces the baseline on Inputs). Option B = EBANX primary + dLocal second MoR through Yuno; its provider cost is the baseline minus the MDR reduction, plus Yuno's flat platform fee and usage in bps on the Net TPV above the included block. Levers: L1 MDR saving (100% contribution), L2 retries and routing, L3 local methods, L4 integrations avoided (per-market EBANX work, later direct integrations, maintenance; deck lever L5), and, kept apart as a 2027 value, L5 time to market (run rate reached by mid 2027 instead of end 2027; deck lever L3). Contribution view nets the take rate and processing cost on incremental GMV. Yuno-wide figures used only as guardrails: 7% authorization uplift, 30% recovered revenue (y.uno).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="30">
+    <mergeCell ref="B37:G40"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B31:C31"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B12:C12"/>
@@ -1172,14 +1330,20 @@
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B34:C34"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B28:G31"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1191,7 +1355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1805,17 +1969,17 @@
         </is>
       </c>
       <c r="D25" s="31" t="n">
-        <v>0.005</v>
+        <v>0.02</v>
       </c>
       <c r="E25" s="31" t="n">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
       <c r="F25" s="31" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="G25" s="28" t="inlineStr">
         <is>
-          <t>ESTIMATE. Methods carried through Yuno via dLocal and not on the EBANX connection (docs.y.uno Payment Type list, 14 Oct 2026): Argentina MODO, Rapipago, Pago Facil; Colombia Bre-B, Nequi, PSE, Efecty; Bolivia Multipago, Pago al Paso; Mexico CoDi, Paynet, 7-Eleven. Context: Pix = 42% of Brazil e-commerce value in 2025 (Worldpay GPR 2026 via Poder360); account-to-account 15% and wallets 39% of Argentina e-commerce value 2025 (GPR 2026 via LetsMoney); QR = 36% of payments in Bolivia in 2025 (Banco Central de Bolivia via Los Tiempos, Jun 2026). EBANX direct coverage per country TO VALIDATE against its quote.</t>
+          <t>ESTIMATE, +2 / +4 / +6% of sales (German, 15 Oct 2026: LatAm is APM-driven). Basis: Pix is 42% of online purchases in Brazil, PSE 64% of e-commerce transactions in Colombia, wallets 46% of e-commerce in Argentina (German, 15 Oct 2026). Through Yuno the checkout adds the methods a single provider does not carry (MODO and interoperable QR in Argentina, Bre-B and Nequi in Colombia, cards and QR in Bolivia) and optimizes the method mix per market. Methods carried through Yuno via dLocal and not on the EBANX connection (docs.y.uno Payment Type list, 14 Oct 2026): Argentina MODO, Rapipago, Pago Facil; Colombia Bre-B, Nequi, PSE, Efecty; Bolivia Multipago, Pago al Paso; Mexico CoDi, Paynet, 7-Eleven. Context: Pix = 42% of Brazil e-commerce value in 2025 (Worldpay GPR 2026 via Poder360); account-to-account 15% and wallets 39% of Argentina e-commerce value 2025 (GPR 2026 via LetsMoney); QR = 36% of payments in Bolivia in 2025 (Banco Central de Bolivia via Los Tiempos, Jun 2026). EBANX direct coverage per country TO VALIDATE against its quote.</t>
         </is>
       </c>
       <c r="H25" s="28" t="inlineStr">
@@ -1827,7 +1991,7 @@
     <row r="26">
       <c r="B26" s="24" t="inlineStr">
         <is>
-          <t>6 · Lever 4 (deck L2) · Integrations avoided: per-market EBANX work, later direct integrations, maintenance</t>
+          <t>6 · Lever 4 (deck L5) · Integrations avoided: per-market EBANX work, later direct integrations, maintenance</t>
         </is>
       </c>
       <c r="C26" s="25" t="n"/>
@@ -2502,7 +2666,7 @@
     <row r="49">
       <c r="B49" s="24" t="inlineStr">
         <is>
-          <t>9 · INTERNAL launch lever (switch, default 0 = off; delete this section before the file leaves Yuno)</t>
+          <t>9 · Lever 5 (deck L3) · Time to market: run rate reached sooner (2027 value, kept apart from the recurring levers)</t>
         </is>
       </c>
       <c r="C49" s="25" t="n"/>
@@ -2512,85 +2676,63 @@
       <c r="G49" s="25" t="n"/>
       <c r="H49" s="25" t="n"/>
     </row>
-    <row r="50" ht="30" customHeight="1">
+    <row r="50" ht="45" customHeight="1">
       <c r="B50" s="10" t="inlineStr">
         <is>
+          <t>Through Yuno: months after Dec 2026 to reach the run rate (9 = Sep 2027, 6 = Jun 2027, 4 = Apr 2027), then flat</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D50" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="E50" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="F50" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="G50" s="28" t="inlineStr">
+        <is>
+          <t>Yuno estimate. Through Yuno all five markets go live together on one integration, each with its local methods and more than one provider, so the Shop reaches Cordel's $4 to 5M a month (modelled $4.5M) by mid 2027. Going direct with EBANX, markets are enabled one by one, so the ramp runs linearly from tier 1 in Dec 2026 to tier 4 in Dec 2027 (the ramp months above). Value = extra GMV in 2027 x (take rate minus Option B all-in processing % at run rate). A one-off 2027 value, never added to the recurring a-year totals.</t>
+        </is>
+      </c>
+      <c r="H50" s="28" t="inlineStr">
+        <is>
+          <t>Cordel (volumes by country) · Fatih (launch scope)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="24" t="inlineStr">
+        <is>
+          <t>10 · INTERNAL launch lever (switch, default 0 = off; delete this section before the file leaves Yuno)</t>
+        </is>
+      </c>
+      <c r="C51" s="25" t="n"/>
+      <c r="D51" s="25" t="n"/>
+      <c r="E51" s="25" t="n"/>
+      <c r="F51" s="25" t="n"/>
+      <c r="G51" s="25" t="n"/>
+      <c r="H51" s="25" t="n"/>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="B52" s="10" t="inlineStr">
+        <is>
           <t>Launch credit switch (1 = on, 0 = off)</t>
         </is>
       </c>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="C52" s="26" t="inlineStr">
         <is>
           <t>flag</t>
         </is>
       </c>
-      <c r="D50" s="33" t="n">
+      <c r="D52" s="33" t="n">
         <v>0</v>
-      </c>
-      <c r="E50" s="34">
-        <f>D50</f>
-        <v/>
-      </c>
-      <c r="F50" s="34">
-        <f>D50</f>
-        <v/>
-      </c>
-      <c r="G50" s="28" t="inlineStr">
-        <is>
-          <t>INTERNAL. Optional lever: a monthly credit against the platform fee for the first months after the 1 Dec 2026 billing start. Applies on the Ramp sheet only. Never on the customer slide.</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="inlineStr">
-        <is>
-          <t>Justo · Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>Monthly credit against the platform fee when the switch is on</t>
-        </is>
-      </c>
-      <c r="C51" s="26" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D51" s="41" t="n">
-        <v>3750</v>
-      </c>
-      <c r="E51" s="11">
-        <f>D51</f>
-        <v/>
-      </c>
-      <c r="F51" s="11">
-        <f>D51</f>
-        <v/>
-      </c>
-      <c r="G51" s="28" t="inlineStr">
-        <is>
-          <t>INTERNAL. Credits are allowed against the platform fee only, for named months, written in the contract, no rollover.</t>
-        </is>
-      </c>
-      <c r="H51" s="28" t="inlineStr">
-        <is>
-          <t>Justo · Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="15" customHeight="1">
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>Months the credit applies (from the billing start)</t>
-        </is>
-      </c>
-      <c r="C52" s="26" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="D52" s="33" t="n">
-        <v>3</v>
       </c>
       <c r="E52" s="34">
         <f>D52</f>
@@ -2602,24 +2744,90 @@
       </c>
       <c r="G52" s="28" t="inlineStr">
         <is>
+          <t>INTERNAL. Optional lever: a monthly credit against the platform fee for the first months after the 1 Dec 2026 billing start. Applies on the Ramp sheet only. Never on the customer slide.</t>
+        </is>
+      </c>
+      <c r="H52" s="28" t="inlineStr">
+        <is>
+          <t>Justo · Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Monthly credit against the platform fee when the switch is on</t>
+        </is>
+      </c>
+      <c r="C53" s="26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D53" s="41" t="n">
+        <v>3750</v>
+      </c>
+      <c r="E53" s="11">
+        <f>D53</f>
+        <v/>
+      </c>
+      <c r="F53" s="11">
+        <f>D53</f>
+        <v/>
+      </c>
+      <c r="G53" s="28" t="inlineStr">
+        <is>
+          <t>INTERNAL. Credits are allowed against the platform fee only, for named months, written in the contract, no rollover.</t>
+        </is>
+      </c>
+      <c r="H53" s="28" t="inlineStr">
+        <is>
+          <t>Justo · Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15" customHeight="1">
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Months the credit applies (from the billing start)</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="D54" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="34">
+        <f>D54</f>
+        <v/>
+      </c>
+      <c r="F54" s="34">
+        <f>D54</f>
+        <v/>
+      </c>
+      <c r="G54" s="28" t="inlineStr">
+        <is>
           <t>INTERNAL. Dec 2026 to Feb 2027.</t>
         </is>
       </c>
-      <c r="H52" s="28" t="inlineStr">
+      <c r="H54" s="28" t="inlineStr">
         <is>
           <t>Justo · Finance</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="44" t="inlineStr">
+    <row r="56">
+      <c r="B56" s="44" t="inlineStr">
         <is>
           <t>Published Yuno figures used as guardrails only (never as inputs): 7% authorization uplift and 30% recovered revenue (y.uno). Treat 7% as the ceiling for the optimistic case.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" s="44" t="inlineStr">
+    <row r="57">
+      <c r="B57" s="44" t="inlineStr">
         <is>
           <t>Labels: CONFIRMED (docs.y.uno or y.uno) · PUBLIC DOCS (third-party page, dated) · OPEN (not confirmed in writing, with owner) · ESTIMATE (modeled; assumption stated) · Carry1st estimate (Cordel, Oct 2026).</t>
         </is>
@@ -5429,7 +5637,7 @@
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>L4 (deck L2) · integrations avoided: per-market EBANX work and later integrations over the horizon, plus maintenance, monthly</t>
+          <t>L4 (deck L5) · integrations avoided: per-market EBANX work and later integrations over the horizon, plus maintenance, monthly</t>
         </is>
       </c>
       <c r="B35" s="11">
@@ -13940,7 +14148,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Payback month = first month in which the cumulative net benefit (contribution view) is non-negative. The INTERNAL launch credit switch (Inputs section 9) applies on this sheet only; default off.</t>
+          <t>Payback month = first month in which the cumulative net benefit (contribution view) is non-negative. The INTERNAL launch credit switch (Inputs section 10) applies on this sheet only; default off.</t>
         </is>
       </c>
     </row>
@@ -14177,7 +14385,7 @@
         <v/>
       </c>
       <c r="D12" s="57">
-        <f>IF(AND(Inputs!$E$50=1,1&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,1&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E12" s="57">
@@ -14256,7 +14464,7 @@
         <v/>
       </c>
       <c r="D13" s="57">
-        <f>IF(AND(Inputs!$E$50=1,2&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,2&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E13" s="57">
@@ -14335,7 +14543,7 @@
         <v/>
       </c>
       <c r="D14" s="57">
-        <f>IF(AND(Inputs!$E$50=1,3&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,3&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E14" s="57">
@@ -14414,7 +14622,7 @@
         <v/>
       </c>
       <c r="D15" s="57">
-        <f>IF(AND(Inputs!$E$50=1,4&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,4&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E15" s="57">
@@ -14493,7 +14701,7 @@
         <v/>
       </c>
       <c r="D16" s="57">
-        <f>IF(AND(Inputs!$E$50=1,5&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,5&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E16" s="57">
@@ -14572,7 +14780,7 @@
         <v/>
       </c>
       <c r="D17" s="57">
-        <f>IF(AND(Inputs!$E$50=1,6&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,6&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E17" s="57">
@@ -14651,7 +14859,7 @@
         <v/>
       </c>
       <c r="D18" s="57">
-        <f>IF(AND(Inputs!$E$50=1,7&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,7&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E18" s="57">
@@ -14730,7 +14938,7 @@
         <v/>
       </c>
       <c r="D19" s="57">
-        <f>IF(AND(Inputs!$E$50=1,8&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,8&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E19" s="57">
@@ -14809,7 +15017,7 @@
         <v/>
       </c>
       <c r="D20" s="57">
-        <f>IF(AND(Inputs!$E$50=1,9&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,9&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E20" s="57">
@@ -14888,7 +15096,7 @@
         <v/>
       </c>
       <c r="D21" s="57">
-        <f>IF(AND(Inputs!$E$50=1,10&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,10&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E21" s="57">
@@ -14967,7 +15175,7 @@
         <v/>
       </c>
       <c r="D22" s="57">
-        <f>IF(AND(Inputs!$E$50=1,11&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,11&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E22" s="57">
@@ -15046,7 +15254,7 @@
         <v/>
       </c>
       <c r="D23" s="57">
-        <f>IF(AND(Inputs!$E$50=1,12&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,12&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E23" s="57">
@@ -15125,7 +15333,7 @@
         <v/>
       </c>
       <c r="D24" s="57">
-        <f>IF(AND(Inputs!$E$50=1,13&lt;=Inputs!$E$52),Inputs!$E$51,0)</f>
+        <f>IF(AND(Inputs!$E$52=1,13&lt;=Inputs!$E$54),Inputs!$E$53,0)</f>
         <v/>
       </c>
       <c r="E24" s="57">
@@ -15267,6 +15475,906 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Time to market · going direct (markets enabled one by one, run rate in Dec 2027) vs through Yuno (all five markets live together, run rate by mid 2027)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Monthly sales (Net TPV). Direct: linear from tier 1 in Dec 2026 to tier 4 in Dec 2027. Yuno: linear from tier 1 to tier 4 by the run-rate month on Inputs, then flat. Value = extra 2027 sales x (take rate minus Option B all-in % at run rate). One-off 2027 value, kept apart from the recurring levers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="9.75" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Months after Dec 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Going direct, sales</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Through Yuno, sales</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Extra sales</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Through Yuno, sales</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Extra sales</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Through Yuno, sales</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Extra sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B7/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D7" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B7,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E7" s="59">
+        <f>D7-C7</f>
+        <v/>
+      </c>
+      <c r="F7" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B7,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G7" s="59">
+        <f>F7-C7</f>
+        <v/>
+      </c>
+      <c r="H7" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B7,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I7" s="59">
+        <f>H7-C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Jan 2027</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B8/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D8" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B8,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E8" s="59">
+        <f>D8-C8</f>
+        <v/>
+      </c>
+      <c r="F8" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B8,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G8" s="59">
+        <f>F8-C8</f>
+        <v/>
+      </c>
+      <c r="H8" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B8,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I8" s="59">
+        <f>H8-C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Feb 2027</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B9/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D9" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B9,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E9" s="59">
+        <f>D9-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B9,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G9" s="59">
+        <f>F9-C9</f>
+        <v/>
+      </c>
+      <c r="H9" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B9,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I9" s="59">
+        <f>H9-C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Mar 2027</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B10/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D10" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B10,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E10" s="59">
+        <f>D10-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B10,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G10" s="59">
+        <f>F10-C10</f>
+        <v/>
+      </c>
+      <c r="H10" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B10,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I10" s="59">
+        <f>H10-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Apr 2027</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B11/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D11" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B11,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E11" s="59">
+        <f>D11-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B11,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G11" s="59">
+        <f>F11-C11</f>
+        <v/>
+      </c>
+      <c r="H11" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B11,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I11" s="59">
+        <f>H11-C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>May 2027</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B12/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D12" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B12,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E12" s="59">
+        <f>D12-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B12,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G12" s="59">
+        <f>F12-C12</f>
+        <v/>
+      </c>
+      <c r="H12" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B12,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I12" s="59">
+        <f>H12-C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Jun 2027</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B13/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D13" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B13,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E13" s="59">
+        <f>D13-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B13,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G13" s="59">
+        <f>F13-C13</f>
+        <v/>
+      </c>
+      <c r="H13" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B13,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I13" s="59">
+        <f>H13-C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Jul 2027</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B14/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D14" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B14,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E14" s="59">
+        <f>D14-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B14,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G14" s="59">
+        <f>F14-C14</f>
+        <v/>
+      </c>
+      <c r="H14" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B14,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I14" s="59">
+        <f>H14-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Aug 2027</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B15/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D15" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B15,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E15" s="59">
+        <f>D15-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B15,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G15" s="59">
+        <f>F15-C15</f>
+        <v/>
+      </c>
+      <c r="H15" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B15,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I15" s="59">
+        <f>H15-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Sep 2027</t>
+        </is>
+      </c>
+      <c r="B16" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B16/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D16" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B16,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E16" s="59">
+        <f>D16-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B16,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G16" s="59">
+        <f>F16-C16</f>
+        <v/>
+      </c>
+      <c r="H16" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B16,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I16" s="59">
+        <f>H16-C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Oct 2027</t>
+        </is>
+      </c>
+      <c r="B17" s="60" t="n">
+        <v>10</v>
+      </c>
+      <c r="C17" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B17/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D17" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B17,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E17" s="59">
+        <f>D17-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B17,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G17" s="59">
+        <f>F17-C17</f>
+        <v/>
+      </c>
+      <c r="H17" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B17,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I17" s="59">
+        <f>H17-C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Nov 2027</t>
+        </is>
+      </c>
+      <c r="B18" s="60" t="n">
+        <v>11</v>
+      </c>
+      <c r="C18" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B18/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D18" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B18,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E18" s="59">
+        <f>D18-C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B18,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G18" s="59">
+        <f>F18-C18</f>
+        <v/>
+      </c>
+      <c r="H18" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B18,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I18" s="59">
+        <f>H18-C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Dec 2027</t>
+        </is>
+      </c>
+      <c r="B19" s="60" t="n">
+        <v>12</v>
+      </c>
+      <c r="C19" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*B19/(Inputs!$E$48-1)</f>
+        <v/>
+      </c>
+      <c r="D19" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B19,Inputs!$D$50)/Inputs!$D$50</f>
+        <v/>
+      </c>
+      <c r="E19" s="59">
+        <f>D19-C19</f>
+        <v/>
+      </c>
+      <c r="F19" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B19,Inputs!$E$50)/Inputs!$E$50</f>
+        <v/>
+      </c>
+      <c r="G19" s="59">
+        <f>F19-C19</f>
+        <v/>
+      </c>
+      <c r="H19" s="57">
+        <f>Inputs!$E$8*Inputs!$E$6+(Inputs!$E$11*Inputs!$E$6-Inputs!$E$8*Inputs!$E$6)*MIN(B19,Inputs!$F$50)/Inputs!$F$50</f>
+        <v/>
+      </c>
+      <c r="I19" s="59">
+        <f>H19-C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="63" t="inlineStr">
+        <is>
+          <t>Total 2027 (Jan to Dec)</t>
+        </is>
+      </c>
+      <c r="C20" s="65">
+        <f>SUM(C8:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="65">
+        <f>SUM(D8:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="65">
+        <f>SUM(E8:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="65">
+        <f>SUM(F8:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="65">
+        <f>SUM(G8:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="65">
+        <f>SUM(H8:H19)</f>
+        <v/>
+      </c>
+      <c r="I20" s="65">
+        <f>SUM(I8:I19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Optimistic</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Through Yuno: run-rate month</t>
+        </is>
+      </c>
+      <c r="B23" s="22">
+        <f>INDEX($A$7:$A$19,Inputs!$D$50+1)</f>
+        <v/>
+      </c>
+      <c r="C23" s="22">
+        <f>INDEX($A$7:$A$19,Inputs!$E$50+1)</f>
+        <v/>
+      </c>
+      <c r="D23" s="22">
+        <f>INDEX($A$7:$A$19,Inputs!$F$50+1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Extra sales in 2027 (GMV)</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>E20</f>
+        <v/>
+      </c>
+      <c r="C24" s="11">
+        <f>G20</f>
+        <v/>
+      </c>
+      <c r="D24" s="11">
+        <f>I20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Option B all-in processing, % of sales at run rate</t>
+        </is>
+      </c>
+      <c r="B25" s="46">
+        <f>Model!E27</f>
+        <v/>
+      </c>
+      <c r="C25" s="46">
+        <f>Model!I27</f>
+        <v/>
+      </c>
+      <c r="D25" s="46">
+        <f>Model!M27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Contribution per $1 of extra sales (take rate minus processing)</t>
+        </is>
+      </c>
+      <c r="B26" s="36">
+        <f>Inputs!$D$13-Inputs!$D$14*B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="36">
+        <f>Inputs!$E$13-Inputs!$E$14*C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="36">
+        <f>Inputs!$F$13-Inputs!$F$14*D25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>L5 (deck L3) · time to market, 2027 value from reaching run rate sooner</t>
+        </is>
+      </c>
+      <c r="B27" s="16">
+        <f>B24*B26</f>
+        <v/>
+      </c>
+      <c r="C27" s="16">
+        <f>C24*C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="16">
+        <f>D24*D26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Recurring levers L1 to L4, a year at run rate (gross, contribution)</t>
+        </is>
+      </c>
+      <c r="B28" s="45">
+        <f>Model!E47</f>
+        <v/>
+      </c>
+      <c r="C28" s="45">
+        <f>Model!I47</f>
+        <v/>
+      </c>
+      <c r="D28" s="45">
+        <f>Model!M47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>2027 value including time to market (recurring + L5)</t>
+        </is>
+      </c>
+      <c r="B29" s="16">
+        <f>B28+B27</f>
+        <v/>
+      </c>
+      <c r="C29" s="16">
+        <f>C28+C27</f>
+        <v/>
+      </c>
+      <c r="D29" s="16">
+        <f>D28+D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Yuno cost a year at run rate</t>
+        </is>
+      </c>
+      <c r="B30" s="45">
+        <f>Model!E46</f>
+        <v/>
+      </c>
+      <c r="C30" s="45">
+        <f>Model!I46</f>
+        <v/>
+      </c>
+      <c r="D30" s="45">
+        <f>Model!M46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Net a year, recurring levers only</t>
+        </is>
+      </c>
+      <c r="B31" s="11">
+        <f>B28-B30</f>
+        <v/>
+      </c>
+      <c r="C31" s="11">
+        <f>C28-C30</f>
+        <v/>
+      </c>
+      <c r="D31" s="11">
+        <f>D28-D30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>Net, 2027 value including time to market</t>
+        </is>
+      </c>
+      <c r="B32" s="16">
+        <f>B29-B30</f>
+        <v/>
+      </c>
+      <c r="C32" s="16">
+        <f>C29-C30</f>
+        <v/>
+      </c>
+      <c r="D32" s="16">
+        <f>D29-D30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>Recurring levers / Yuno cost</t>
+        </is>
+      </c>
+      <c r="B33" s="20">
+        <f>B28/B30</f>
+        <v/>
+      </c>
+      <c r="C33" s="20">
+        <f>C28/C30</f>
+        <v/>
+      </c>
+      <c r="D33" s="20">
+        <f>D28/D30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>2027 value including time to market / Yuno cost</t>
+        </is>
+      </c>
+      <c r="B34" s="20">
+        <f>B29/B30</f>
+        <v/>
+      </c>
+      <c r="C34" s="20">
+        <f>C29/C30</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>D29/D30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>L5 is value in the first year from reaching scale sooner: shown as a 2027 figure and never added to the recurring a-year totals. Ramp shapes are Yuno ESTIMATES; replace with Cordel's written projections by country.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="H5:I5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -16293,7 +17401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
carry1st: integrations lever raised (dev cost above $150K a year) in model and both decks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Carry1st/build/model/bc_model.xlsx
+++ b/Deals/Carry1st/build/model/bc_model.xlsx
@@ -2046,13 +2046,13 @@
         </is>
       </c>
       <c r="D28" s="38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" s="38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F28" s="38" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G28" s="28" t="inlineStr">
         <is>
@@ -2077,13 +2077,13 @@
         </is>
       </c>
       <c r="D29" s="38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" s="38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29" s="38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G29" s="28" t="inlineStr">
         <is>
@@ -2108,13 +2108,13 @@
         </is>
       </c>
       <c r="D30" s="38" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E30" s="38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F30" s="38" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G30" s="28" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="D31" s="39" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="E31" s="11">
         <f>D31</f>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="G31" s="28" t="inlineStr">
         <is>
-          <t>ESTIMATE, about $104K a year loaded. Sits between Cape Town senior engineer market pay (PayScale, 2026; Carry1st engineers are in Cape Town) and LatAm loaded cost of $87.5K to $100.8K a year (Second Talent, 2026); US fully loaded is $200K to $280K (Revelo, 2026).</t>
+          <t>ESTIMATE, $130K a year loaded: a senior payments engineer (Justo, 15 Oct 2026: incremental dev cost avoided above $150K a year). Above LatAm loaded cost of $87.5K to $100.8K a year (Second Talent, 2026), below US fully loaded $200K to $280K (Revelo, 2026).</t>
         </is>
       </c>
       <c r="H31" s="28" t="inlineStr">
@@ -2172,13 +2172,13 @@
         </is>
       </c>
       <c r="D32" s="40" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="E32" s="40" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="F32" s="40" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="G32" s="28" t="inlineStr">
         <is>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="G33" s="28" t="inlineStr">
         <is>
-          <t>52 weeks x $2,000 = $104K a year loaded per FTE.</t>
+          <t>52 weeks x $2,500 = $130K a year loaded per FTE.</t>
         </is>
       </c>
       <c r="H33" s="28" t="inlineStr"/>

</xml_diff>

<commit_message>
carry1st: time-to-market lever more conservative (run rate Oct/Aug/Jul 2027: $411K / $843K / $1.08M), both decks and model
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Carry1st/build/model/bc_model.xlsx
+++ b/Deals/Carry1st/build/model/bc_model.xlsx
@@ -2688,13 +2688,13 @@
         </is>
       </c>
       <c r="D50" s="38" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E50" s="38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F50" s="38" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G50" s="28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
carry1st: time-to-market lever lowered again (Nov/Sep/Aug 2027: $206K / $632K / $863K)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Deals/Carry1st/build/model/bc_model.xlsx
+++ b/Deals/Carry1st/build/model/bc_model.xlsx
@@ -2688,13 +2688,13 @@
         </is>
       </c>
       <c r="D50" s="38" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E50" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="F50" s="38" t="n">
         <v>8</v>
-      </c>
-      <c r="F50" s="38" t="n">
-        <v>7</v>
       </c>
       <c r="G50" s="28" t="inlineStr">
         <is>

</xml_diff>